<commit_message>
refactor of entities and relationships to be named under Model
</commit_message>
<xml_diff>
--- a/mappings/data_domains_template.xlsx
+++ b/mappings/data_domains_template.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="53">
   <si>
     <t xml:space="preserve">DomainNamespace</t>
   </si>
@@ -131,6 +131,57 @@
   </si>
   <si>
     <t xml:space="preserve">XML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORACLEDATATYPES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VARCHAR2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NUMBER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RAW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XMLTYPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LONG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NVARCHAR2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROWID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BLOB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LONG RAW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNDEFINED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANYDATA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLOAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BFILE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NCLOB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INTERVAL</t>
   </si>
 </sst>
 </file>
@@ -373,7 +424,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AT61"/>
+  <dimension ref="A1:AT48"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.51"/>
@@ -711,10 +762,10 @@
       <c r="A21" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -722,10 +773,10 @@
       <c r="A22" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -733,10 +784,10 @@
       <c r="A23" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" s="1" t="s">
         <v>29</v>
       </c>
     </row>
@@ -744,10 +795,10 @@
       <c r="A24" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C24" s="1" t="s">
         <v>30</v>
       </c>
     </row>
@@ -755,10 +806,10 @@
       <c r="A25" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="C25" s="1" t="s">
         <v>31</v>
       </c>
     </row>
@@ -766,10 +817,10 @@
       <c r="A26" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="C26" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -777,10 +828,10 @@
       <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="C27" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -788,10 +839,10 @@
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="C28" s="1" t="s">
         <v>34</v>
       </c>
     </row>
@@ -799,108 +850,221 @@
       <c r="A29" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="C29" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="0"/>
+      <c r="A30" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="0"/>
+      <c r="A31" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="0"/>
+      <c r="A32" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="0"/>
+      <c r="A33" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="0"/>
+      <c r="A34" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="0"/>
+      <c r="A35" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="0"/>
+      <c r="A36" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="0"/>
+      <c r="A37" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="0"/>
+      <c r="A38" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="0"/>
+      <c r="A39" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="0"/>
+      <c r="A40" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="0"/>
+      <c r="A41" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="0"/>
+      <c r="A42" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="0"/>
+      <c r="A43" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="0"/>
+      <c r="A44" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="0"/>
+      <c r="A45" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="0"/>
+      <c r="A46" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="0"/>
+      <c r="A47" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="0"/>
-    </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="0"/>
-    </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="0"/>
-    </row>
-    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="0"/>
-    </row>
-    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="0"/>
-    </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="0"/>
-    </row>
-    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="0"/>
-    </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="0"/>
-    </row>
-    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="0"/>
-    </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="0"/>
-    </row>
-    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="0"/>
-    </row>
-    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="0"/>
-    </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="0"/>
-    </row>
-    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="0"/>
+      <c r="A48" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>52</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:B47"/>

</xml_diff>